<commit_message>
add name in xlsx file
</commit_message>
<xml_diff>
--- a/lab3_JUnit/Testcase_Template_673380262-4.xlsx
+++ b/lab3_JUnit/Testcase_Template_673380262-4.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="93">
   <si>
     <t>Use case ID/ Req. ID</t>
   </si>
@@ -239,6 +239,9 @@
   </si>
   <si>
     <t xml:space="preserve">Designer: ระบุชื่อนามสกุล รหัสนักศึกษา </t>
+  </si>
+  <si>
+    <t>กรมภัฏ พิริยะ 673380262-4</t>
   </si>
   <si>
     <t xml:space="preserve">Test Environtment: </t>
@@ -527,7 +530,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -655,6 +658,9 @@
     </xf>
     <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -31785,7 +31791,9 @@
       <c r="E5" s="52" t="s">
         <v>72</v>
       </c>
-      <c r="F5" s="53"/>
+      <c r="F5" s="54" t="s">
+        <v>73</v>
+      </c>
       <c r="G5" s="12"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -31808,10 +31816,10 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6" ht="24.0" customHeight="1">
-      <c r="A6" s="54" t="s">
-        <v>73</v>
+      <c r="A6" s="55" t="s">
+        <v>74</v>
       </c>
-      <c r="B6" s="55"/>
+      <c r="B6" s="56"/>
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
@@ -31866,86 +31874,86 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" ht="24.0" customHeight="1">
-      <c r="A8" s="56" t="s">
+      <c r="A8" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="56" t="s">
-        <v>74</v>
+      <c r="B8" s="57" t="s">
+        <v>75</v>
       </c>
-      <c r="C8" s="57" t="s">
+      <c r="C8" s="58" t="s">
         <v>50</v>
       </c>
       <c r="D8" s="12"/>
-      <c r="E8" s="56" t="s">
-        <v>75</v>
-      </c>
-      <c r="F8" s="56" t="s">
+      <c r="E8" s="57" t="s">
         <v>76</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="F8" s="57" t="s">
         <v>77</v>
       </c>
-      <c r="H8" s="58"/>
-      <c r="I8" s="58"/>
-      <c r="J8" s="58"/>
-      <c r="K8" s="58"/>
-      <c r="L8" s="58"/>
-      <c r="M8" s="58"/>
-      <c r="N8" s="58"/>
-      <c r="O8" s="58"/>
-      <c r="P8" s="58"/>
-      <c r="Q8" s="58"/>
-      <c r="R8" s="58"/>
-      <c r="S8" s="58"/>
-      <c r="T8" s="58"/>
-      <c r="U8" s="58"/>
-      <c r="V8" s="58"/>
-      <c r="W8" s="58"/>
-      <c r="X8" s="58"/>
-      <c r="Y8" s="58"/>
-      <c r="Z8" s="58"/>
+      <c r="G8" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="H8" s="59"/>
+      <c r="I8" s="59"/>
+      <c r="J8" s="59"/>
+      <c r="K8" s="59"/>
+      <c r="L8" s="59"/>
+      <c r="M8" s="59"/>
+      <c r="N8" s="59"/>
+      <c r="O8" s="59"/>
+      <c r="P8" s="59"/>
+      <c r="Q8" s="59"/>
+      <c r="R8" s="59"/>
+      <c r="S8" s="59"/>
+      <c r="T8" s="59"/>
+      <c r="U8" s="59"/>
+      <c r="V8" s="59"/>
+      <c r="W8" s="59"/>
+      <c r="X8" s="59"/>
+      <c r="Y8" s="59"/>
+      <c r="Z8" s="59"/>
     </row>
     <row r="9" ht="24.0" customHeight="1">
       <c r="A9" s="40"/>
       <c r="B9" s="40"/>
-      <c r="C9" s="59" t="s">
-        <v>78</v>
+      <c r="C9" s="60" t="s">
+        <v>79</v>
       </c>
-      <c r="D9" s="59" t="s">
-        <v>79</v>
+      <c r="D9" s="60" t="s">
+        <v>80</v>
       </c>
       <c r="E9" s="40"/>
       <c r="F9" s="40"/>
-      <c r="G9" s="60"/>
-      <c r="H9" s="58"/>
-      <c r="I9" s="58"/>
-      <c r="J9" s="58"/>
-      <c r="K9" s="58"/>
-      <c r="L9" s="58"/>
-      <c r="M9" s="58"/>
-      <c r="N9" s="58"/>
-      <c r="O9" s="58"/>
-      <c r="P9" s="58"/>
-      <c r="Q9" s="58"/>
-      <c r="R9" s="58"/>
-      <c r="S9" s="58"/>
-      <c r="T9" s="58"/>
-      <c r="U9" s="58"/>
-      <c r="V9" s="58"/>
-      <c r="W9" s="58"/>
-      <c r="X9" s="58"/>
-      <c r="Y9" s="58"/>
-      <c r="Z9" s="58"/>
+      <c r="G9" s="61"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="59"/>
+      <c r="J9" s="59"/>
+      <c r="K9" s="59"/>
+      <c r="L9" s="59"/>
+      <c r="M9" s="59"/>
+      <c r="N9" s="59"/>
+      <c r="O9" s="59"/>
+      <c r="P9" s="59"/>
+      <c r="Q9" s="59"/>
+      <c r="R9" s="59"/>
+      <c r="S9" s="59"/>
+      <c r="T9" s="59"/>
+      <c r="U9" s="59"/>
+      <c r="V9" s="59"/>
+      <c r="W9" s="59"/>
+      <c r="X9" s="59"/>
+      <c r="Y9" s="59"/>
+      <c r="Z9" s="59"/>
     </row>
     <row r="10" ht="24.0" customHeight="1">
-      <c r="A10" s="61" t="s">
+      <c r="A10" s="62" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D10" s="9">
         <v>3.0</v>
@@ -31982,16 +31990,16 @@
     <row r="11" ht="24.0" customHeight="1">
       <c r="A11" s="38"/>
       <c r="B11" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D11" s="9">
         <v>3.0</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F11" s="13" t="s">
         <v>62</v>
@@ -32022,19 +32030,19 @@
     <row r="12" ht="24.0" customHeight="1">
       <c r="A12" s="38"/>
       <c r="B12" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D12" s="13">
         <v>0.0</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G12" s="13" t="s">
         <v>4</v>
@@ -32062,7 +32070,7 @@
     <row r="13" ht="24.0" customHeight="1">
       <c r="A13" s="40"/>
       <c r="B13" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C13" s="13">
         <v>4567.0</v>
@@ -32071,7 +32079,7 @@
         <v>0.0</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>62</v>
@@ -32105,11 +32113,11 @@
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="62" t="s">
-        <v>90</v>
+      <c r="F14" s="63" t="s">
+        <v>91</v>
       </c>
-      <c r="G14" s="62" t="s">
-        <v>90</v>
+      <c r="G14" s="63" t="s">
+        <v>91</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
@@ -32138,8 +32146,8 @@
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
-      <c r="G15" s="62" t="s">
-        <v>91</v>
+      <c r="G15" s="63" t="s">
+        <v>92</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>

</xml_diff>